<commit_message>
docs: Switch to cover page.
</commit_message>
<xml_diff>
--- a/Income And Expenses Forecast Demo.xlsx
+++ b/Income And Expenses Forecast Demo.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowHeight="22160" activeTab="2"/>
+    <workbookView windowHeight="22160"/>
   </bookViews>
   <sheets>
     <sheet name="Cover Page" sheetId="18" r:id="rId1"/>
@@ -39203,7 +39203,7 @@
       <c r="H50" s="14"/>
       <c r="I50" s="48"/>
     </row>
-    <row r="51" ht="34" spans="1:9">
+    <row r="51" spans="1:9">
       <c r="A51" s="38" t="str" cm="1">
         <f ca="1" t="array" ref="A51">IF((INDIRECT("'"&amp;INDIRECT("Main!B9")&amp;"'!A65"))=0,"",(INDIRECT("'"&amp;INDIRECT("Main!B9")&amp;"'!A65")))</f>
         <v>Birdie Sim Card</v>

</xml_diff>

<commit_message>
docs: 1. Update Assets. 2. Update Expenses.
</commit_message>
<xml_diff>
--- a/Income And Expenses Forecast Demo.xlsx
+++ b/Income And Expenses Forecast Demo.xlsx
@@ -425,7 +425,9 @@
 ~Oxford Dictionary $19.99 (Don't Need To Include)
 ~Round Trip to the East Kowloon hospital ~ $4
 ~KFC ~ $31
-~Shu Shi (Chuk Yuen Plaza) ~ $98</t>
+~Shu Shi (Chuk Yuen Plaza) ~ $98
+~ Coin Machine Transaction Fees ~ $2.7
+~ Best Mart 360 ~ $18</t>
   </si>
   <si>
     <t xml:space="preserve">~ Payback $570 to Mom </t>
@@ -4790,7 +4792,7 @@
       </c>
       <c r="C2" s="4" cm="1">
         <f ca="1" t="array" ref="C2">INDIRECT("'"&amp;Main!B9&amp;"'!$C$16")</f>
-        <v>78.22</v>
+        <v>57.52</v>
       </c>
       <c r="D2" s="4"/>
       <c r="E2" s="4"/>
@@ -4806,7 +4808,7 @@
       </c>
       <c r="C3" s="7">
         <f ca="1">E190</f>
-        <v>8468.42000000001</v>
+        <v>8447.72</v>
       </c>
       <c r="D3" s="7"/>
       <c r="E3" s="7"/>
@@ -4822,7 +4824,7 @@
       <c r="B4" s="9"/>
       <c r="C4" s="10">
         <f ca="1">SUM(C2:G3)</f>
-        <v>8546.64</v>
+        <v>8505.24000000001</v>
       </c>
       <c r="D4" s="10"/>
       <c r="E4" s="10"/>
@@ -6643,7 +6645,7 @@
       <c r="D116" s="58"/>
       <c r="E116" s="71" cm="1">
         <f ca="1" t="array" ref="E116">INDIRECT("'"&amp;INDIRECT("Main!B27")&amp;"'!E190")</f>
-        <v>6632.39</v>
+        <v>6611.69</v>
       </c>
       <c r="F116" s="14"/>
       <c r="G116" s="14"/>
@@ -6915,7 +6917,7 @@
       <c r="D136" s="82"/>
       <c r="E136" s="89">
         <f ca="1">(F16+E116)-(SUM(E118:E127)+SUM(E129:E135))</f>
-        <v>7207.40000000001</v>
+        <v>7186.7</v>
       </c>
       <c r="F136" s="14"/>
       <c r="G136" s="14"/>
@@ -7007,7 +7009,7 @@
       <c r="D143" s="58"/>
       <c r="E143" s="89">
         <f ca="1">E136</f>
-        <v>7207.40000000001</v>
+        <v>7186.7</v>
       </c>
       <c r="F143" s="14"/>
       <c r="G143" s="14"/>
@@ -7279,7 +7281,7 @@
       <c r="D163" s="82"/>
       <c r="E163" s="92">
         <f ca="1">(F28+E143)-(SUM(E145:E154)+SUM(E156:E162))</f>
-        <v>7893.41000000001</v>
+        <v>7872.71</v>
       </c>
       <c r="F163" s="14"/>
       <c r="G163" s="14"/>
@@ -7371,7 +7373,7 @@
       <c r="D170" s="58"/>
       <c r="E170" s="92">
         <f ca="1">E163</f>
-        <v>7893.41000000001</v>
+        <v>7872.71</v>
       </c>
       <c r="F170" s="14"/>
       <c r="G170" s="14"/>
@@ -7643,7 +7645,7 @@
       <c r="D190" s="82"/>
       <c r="E190" s="92">
         <f ca="1">(F40+E170)-(SUM(E172:E181)+SUM(E183:E189))</f>
-        <v>8468.42000000001</v>
+        <v>8447.72</v>
       </c>
       <c r="F190" s="14"/>
       <c r="G190" s="14"/>
@@ -8154,7 +8156,7 @@
       </c>
       <c r="C2" s="4" cm="1">
         <f ca="1" t="array" ref="C2">INDIRECT("'"&amp;Main!B9&amp;"'!$C$16")</f>
-        <v>78.22</v>
+        <v>57.52</v>
       </c>
       <c r="D2" s="4"/>
       <c r="E2" s="4"/>
@@ -8170,7 +8172,7 @@
       </c>
       <c r="C3" s="7">
         <f ca="1">E190</f>
-        <v>10575.45</v>
+        <v>10554.75</v>
       </c>
       <c r="D3" s="7"/>
       <c r="E3" s="7"/>
@@ -8186,7 +8188,7 @@
       <c r="B4" s="9"/>
       <c r="C4" s="10">
         <f ca="1">SUM(C2:G3)</f>
-        <v>10653.67</v>
+        <v>10612.27</v>
       </c>
       <c r="D4" s="10"/>
       <c r="E4" s="10"/>
@@ -10007,7 +10009,7 @@
       <c r="D116" s="58"/>
       <c r="E116" s="71" cm="1">
         <f ca="1" t="array" ref="E116">INDIRECT("'"&amp;INDIRECT("Main!B30")&amp;"'!E190")</f>
-        <v>8468.42000000001</v>
+        <v>8447.72</v>
       </c>
       <c r="F116" s="14"/>
       <c r="G116" s="14"/>
@@ -10279,7 +10281,7 @@
       <c r="D136" s="82"/>
       <c r="E136" s="89">
         <f ca="1">(F16+E116)-(SUM(E118:E127)+SUM(E129:E135))</f>
-        <v>9314.43000000001</v>
+        <v>9293.73</v>
       </c>
       <c r="F136" s="14"/>
       <c r="G136" s="14"/>
@@ -10371,7 +10373,7 @@
       <c r="D143" s="58"/>
       <c r="E143" s="89">
         <f ca="1">E136</f>
-        <v>9314.43000000001</v>
+        <v>9293.73</v>
       </c>
       <c r="F143" s="14"/>
       <c r="G143" s="14"/>
@@ -10643,7 +10645,7 @@
       <c r="D163" s="82"/>
       <c r="E163" s="92">
         <f ca="1">(F28+E143)-(SUM(E145:E154)+SUM(E156:E162))</f>
-        <v>9729.44000000001</v>
+        <v>9708.74000000001</v>
       </c>
       <c r="F163" s="14"/>
       <c r="G163" s="14"/>
@@ -10735,7 +10737,7 @@
       <c r="D170" s="58"/>
       <c r="E170" s="92">
         <f ca="1">E163</f>
-        <v>9729.44000000001</v>
+        <v>9708.74000000001</v>
       </c>
       <c r="F170" s="14"/>
       <c r="G170" s="14"/>
@@ -11007,7 +11009,7 @@
       <c r="D190" s="82"/>
       <c r="E190" s="92">
         <f ca="1">(F40+E170)-(SUM(E172:E181)+SUM(E183:E189))</f>
-        <v>10575.45</v>
+        <v>10554.75</v>
       </c>
       <c r="F190" s="14"/>
       <c r="G190" s="14"/>
@@ -11514,7 +11516,7 @@
       </c>
       <c r="C2" s="4" cm="1">
         <f ca="1" t="array" ref="C2">INDIRECT("'"&amp;Main!B9&amp;"'!$C$16")</f>
-        <v>78.22</v>
+        <v>57.52</v>
       </c>
       <c r="D2" s="4"/>
       <c r="E2" s="4"/>
@@ -11530,7 +11532,7 @@
       </c>
       <c r="C3" s="7">
         <f ca="1">E190</f>
-        <v>14875.45</v>
+        <v>14854.75</v>
       </c>
       <c r="D3" s="7"/>
       <c r="E3" s="7"/>
@@ -11546,7 +11548,7 @@
       <c r="B4" s="9"/>
       <c r="C4" s="10">
         <f ca="1">SUM(C2:G3)</f>
-        <v>14953.67</v>
+        <v>14912.27</v>
       </c>
       <c r="D4" s="10"/>
       <c r="E4" s="10"/>
@@ -13371,7 +13373,7 @@
       <c r="D116" s="58"/>
       <c r="E116" s="71" cm="1">
         <f ca="1" t="array" ref="E116">INDIRECT("'"&amp;INDIRECT("Main!B33")&amp;"'!E190")</f>
-        <v>10575.45</v>
+        <v>10554.75</v>
       </c>
       <c r="F116" s="14"/>
       <c r="G116" s="14"/>
@@ -13643,7 +13645,7 @@
       <c r="D136" s="82"/>
       <c r="E136" s="89">
         <f ca="1">(F16+E116)-(SUM(E118:E127)+SUM(E129:E135))</f>
-        <v>11791.45</v>
+        <v>11770.75</v>
       </c>
       <c r="F136" s="14"/>
       <c r="G136" s="14"/>
@@ -13735,7 +13737,7 @@
       <c r="D143" s="58"/>
       <c r="E143" s="89">
         <f ca="1">E136</f>
-        <v>11791.45</v>
+        <v>11770.75</v>
       </c>
       <c r="F143" s="14"/>
       <c r="G143" s="14"/>
@@ -14007,7 +14009,7 @@
       <c r="D163" s="82"/>
       <c r="E163" s="92">
         <f ca="1">(F28+E143)-(SUM(E145:E154)+SUM(E156:E162))</f>
-        <v>13659.45</v>
+        <v>13638.75</v>
       </c>
       <c r="F163" s="14"/>
       <c r="G163" s="14"/>
@@ -14099,7 +14101,7 @@
       <c r="D170" s="58"/>
       <c r="E170" s="92">
         <f ca="1">E163</f>
-        <v>13659.45</v>
+        <v>13638.75</v>
       </c>
       <c r="F170" s="14"/>
       <c r="G170" s="14"/>
@@ -14371,7 +14373,7 @@
       <c r="D190" s="82"/>
       <c r="E190" s="92">
         <f ca="1">(F40+E170)-(SUM(E172:E181)+SUM(E183:E189))</f>
-        <v>14875.45</v>
+        <v>14854.75</v>
       </c>
       <c r="F190" s="14"/>
       <c r="G190" s="14"/>
@@ -14876,7 +14878,7 @@
       </c>
       <c r="C2" s="4" cm="1">
         <f ca="1" t="array" ref="C2">INDIRECT("'"&amp;Main!B9&amp;"'!$C$16")</f>
-        <v>78.22</v>
+        <v>57.52</v>
       </c>
       <c r="D2" s="4"/>
       <c r="E2" s="4"/>
@@ -14892,7 +14894,7 @@
       </c>
       <c r="C3" s="7">
         <f ca="1">E190</f>
-        <v>16711.48</v>
+        <v>16690.78</v>
       </c>
       <c r="D3" s="7"/>
       <c r="E3" s="7"/>
@@ -14908,7 +14910,7 @@
       <c r="B4" s="9"/>
       <c r="C4" s="10">
         <f ca="1">SUM(C2:G3)</f>
-        <v>16789.7</v>
+        <v>16748.3</v>
       </c>
       <c r="D4" s="10"/>
       <c r="E4" s="10"/>
@@ -16729,7 +16731,7 @@
       <c r="D116" s="58"/>
       <c r="E116" s="71" cm="1">
         <f ca="1" t="array" ref="E116">INDIRECT("'"&amp;INDIRECT("Main!B36")&amp;"'!E190")</f>
-        <v>14875.45</v>
+        <v>14854.75</v>
       </c>
       <c r="F116" s="14"/>
       <c r="G116" s="14"/>
@@ -17001,7 +17003,7 @@
       <c r="D136" s="82"/>
       <c r="E136" s="89">
         <f ca="1">(F16+E116)-(SUM(E118:E127)+SUM(E129:E135))</f>
-        <v>15450.46</v>
+        <v>15429.76</v>
       </c>
       <c r="F136" s="14"/>
       <c r="G136" s="14"/>
@@ -17093,7 +17095,7 @@
       <c r="D143" s="58"/>
       <c r="E143" s="89">
         <f ca="1">E136</f>
-        <v>15450.46</v>
+        <v>15429.76</v>
       </c>
       <c r="F143" s="14"/>
       <c r="G143" s="14"/>
@@ -17365,7 +17367,7 @@
       <c r="D163" s="82"/>
       <c r="E163" s="92">
         <f ca="1">(F28+E143)-(SUM(E145:E154)+SUM(E156:E162))</f>
-        <v>16136.47</v>
+        <v>16115.77</v>
       </c>
       <c r="F163" s="14"/>
       <c r="G163" s="14"/>
@@ -17457,7 +17459,7 @@
       <c r="D170" s="58"/>
       <c r="E170" s="92">
         <f ca="1">E163</f>
-        <v>16136.47</v>
+        <v>16115.77</v>
       </c>
       <c r="F170" s="14"/>
       <c r="G170" s="14"/>
@@ -17729,7 +17731,7 @@
       <c r="D190" s="82"/>
       <c r="E190" s="92">
         <f ca="1">(F40+E170)-(SUM(E172:E181)+SUM(E183:E189))</f>
-        <v>16711.48</v>
+        <v>16690.78</v>
       </c>
       <c r="F190" s="14"/>
       <c r="G190" s="14"/>
@@ -18241,7 +18243,7 @@
       </c>
       <c r="C2" s="4" cm="1">
         <f ca="1" t="array" ref="C2">INDIRECT("'"&amp;Main!B9&amp;"'!$C$16")</f>
-        <v>78.22</v>
+        <v>57.52</v>
       </c>
       <c r="D2" s="4"/>
       <c r="E2" s="4"/>
@@ -18257,7 +18259,7 @@
       </c>
       <c r="C3" s="7">
         <f ca="1">E190</f>
-        <v>18818.51</v>
+        <v>18797.81</v>
       </c>
       <c r="D3" s="7"/>
       <c r="E3" s="7"/>
@@ -18273,7 +18275,7 @@
       <c r="B4" s="9"/>
       <c r="C4" s="10">
         <f ca="1">SUM(C2:G3)</f>
-        <v>18896.73</v>
+        <v>18855.33</v>
       </c>
       <c r="D4" s="10"/>
       <c r="E4" s="10"/>
@@ -20094,7 +20096,7 @@
       <c r="D116" s="58"/>
       <c r="E116" s="71" cm="1">
         <f ca="1" t="array" ref="E116">INDIRECT("'"&amp;INDIRECT("Main!B39")&amp;"'!E190")</f>
-        <v>16711.48</v>
+        <v>16690.78</v>
       </c>
       <c r="F116" s="14"/>
       <c r="G116" s="14"/>
@@ -20366,7 +20368,7 @@
       <c r="D136" s="82"/>
       <c r="E136" s="89">
         <f ca="1">(F16+E116)-(SUM(E118:E127)+SUM(E129:E135))</f>
-        <v>17557.49</v>
+        <v>17536.79</v>
       </c>
       <c r="F136" s="14"/>
       <c r="G136" s="14"/>
@@ -20458,7 +20460,7 @@
       <c r="D143" s="58"/>
       <c r="E143" s="89">
         <f ca="1">E136</f>
-        <v>17557.49</v>
+        <v>17536.79</v>
       </c>
       <c r="F143" s="14"/>
       <c r="G143" s="14"/>
@@ -20730,7 +20732,7 @@
       <c r="D163" s="82"/>
       <c r="E163" s="92">
         <f ca="1">(F28+E143)-(SUM(E145:E154)+SUM(E156:E162))</f>
-        <v>17972.5</v>
+        <v>17951.8</v>
       </c>
       <c r="F163" s="14"/>
       <c r="G163" s="14"/>
@@ -20822,7 +20824,7 @@
       <c r="D170" s="58"/>
       <c r="E170" s="92">
         <f ca="1">E163</f>
-        <v>17972.5</v>
+        <v>17951.8</v>
       </c>
       <c r="F170" s="14"/>
       <c r="G170" s="14"/>
@@ -21094,7 +21096,7 @@
       <c r="D190" s="82"/>
       <c r="E190" s="92">
         <f ca="1">(F40+E170)-(SUM(E172:E181)+SUM(E183:E189))</f>
-        <v>18818.51</v>
+        <v>18797.81</v>
       </c>
       <c r="F190" s="14"/>
       <c r="G190" s="14"/>
@@ -21599,7 +21601,7 @@
       </c>
       <c r="C2" s="4" cm="1">
         <f ca="1" t="array" ref="C2">INDIRECT("'"&amp;Main!B9&amp;"'!$C$16")</f>
-        <v>78.22</v>
+        <v>57.52</v>
       </c>
       <c r="D2" s="4"/>
       <c r="E2" s="4"/>
@@ -21615,7 +21617,7 @@
       </c>
       <c r="C3" s="7">
         <f ca="1">E190</f>
-        <v>20744.54</v>
+        <v>20723.84</v>
       </c>
       <c r="D3" s="7"/>
       <c r="E3" s="7"/>
@@ -21631,7 +21633,7 @@
       <c r="B4" s="9"/>
       <c r="C4" s="10">
         <f ca="1">SUM(C2:G3)</f>
-        <v>20822.76</v>
+        <v>20781.36</v>
       </c>
       <c r="D4" s="10"/>
       <c r="E4" s="10"/>
@@ -23452,7 +23454,7 @@
       <c r="D116" s="58"/>
       <c r="E116" s="71" cm="1">
         <f ca="1" t="array" ref="E116">INDIRECT("'"&amp;INDIRECT("Main!B42")&amp;"'!E190")</f>
-        <v>18818.51</v>
+        <v>18797.81</v>
       </c>
       <c r="F116" s="14"/>
       <c r="G116" s="14"/>
@@ -23724,7 +23726,7 @@
       <c r="D136" s="82"/>
       <c r="E136" s="89">
         <f ca="1">(F16+E116)-(SUM(E118:E127)+SUM(E129:E135))</f>
-        <v>19443.52</v>
+        <v>19422.82</v>
       </c>
       <c r="F136" s="14"/>
       <c r="G136" s="14"/>
@@ -23816,7 +23818,7 @@
       <c r="D143" s="58"/>
       <c r="E143" s="89">
         <f ca="1">E136</f>
-        <v>19443.52</v>
+        <v>19422.82</v>
       </c>
       <c r="F143" s="14"/>
       <c r="G143" s="14"/>
@@ -24088,7 +24090,7 @@
       <c r="D163" s="82"/>
       <c r="E163" s="92">
         <f ca="1">(F28+E143)-(SUM(E145:E154)+SUM(E156:E162))</f>
-        <v>20129.53</v>
+        <v>20108.83</v>
       </c>
       <c r="F163" s="14"/>
       <c r="G163" s="14"/>
@@ -24180,7 +24182,7 @@
       <c r="D170" s="58"/>
       <c r="E170" s="92">
         <f ca="1">E163</f>
-        <v>20129.53</v>
+        <v>20108.83</v>
       </c>
       <c r="F170" s="14"/>
       <c r="G170" s="14"/>
@@ -24452,7 +24454,7 @@
       <c r="D190" s="82"/>
       <c r="E190" s="92">
         <f ca="1">(F40+E170)-(SUM(E172:E181)+SUM(E183:E189))</f>
-        <v>20744.54</v>
+        <v>20723.84</v>
       </c>
       <c r="F190" s="14"/>
       <c r="G190" s="14"/>
@@ -24963,7 +24965,7 @@
       </c>
       <c r="C2" s="4" cm="1">
         <f ca="1" t="array" ref="C2">INDIRECT("'"&amp;Main!B9&amp;"'!$C$16")</f>
-        <v>78.22</v>
+        <v>57.52</v>
       </c>
       <c r="D2" s="4"/>
       <c r="E2" s="4"/>
@@ -24979,7 +24981,7 @@
       </c>
       <c r="C3" s="7">
         <f ca="1">E190</f>
-        <v>23934.57</v>
+        <v>23913.87</v>
       </c>
       <c r="D3" s="7"/>
       <c r="E3" s="7"/>
@@ -24995,7 +24997,7 @@
       <c r="B4" s="9"/>
       <c r="C4" s="10">
         <f ca="1">SUM(C2:G3)</f>
-        <v>24012.79</v>
+        <v>23971.39</v>
       </c>
       <c r="D4" s="10"/>
       <c r="E4" s="10"/>
@@ -26820,7 +26822,7 @@
       <c r="D116" s="58"/>
       <c r="E116" s="71" cm="1">
         <f ca="1" t="array" ref="E116">INDIRECT("'"&amp;INDIRECT("Main!B45")&amp;"'!E190")</f>
-        <v>20744.54</v>
+        <v>20723.84</v>
       </c>
       <c r="F116" s="14"/>
       <c r="G116" s="14"/>
@@ -27092,7 +27094,7 @@
       <c r="D136" s="82"/>
       <c r="E136" s="89">
         <f ca="1">(F16+E116)-(SUM(E118:E127)+SUM(E129:E135))</f>
-        <v>21590.55</v>
+        <v>21569.85</v>
       </c>
       <c r="F136" s="14"/>
       <c r="G136" s="14"/>
@@ -27184,7 +27186,7 @@
       <c r="D143" s="58"/>
       <c r="E143" s="89">
         <f ca="1">E136</f>
-        <v>21590.55</v>
+        <v>21569.85</v>
       </c>
       <c r="F143" s="14"/>
       <c r="G143" s="14"/>
@@ -27456,7 +27458,7 @@
       <c r="D163" s="82"/>
       <c r="E163" s="92">
         <f ca="1">(F28+E143)-(SUM(E145:E154)+SUM(E156:E162))</f>
-        <v>23088.56</v>
+        <v>23067.86</v>
       </c>
       <c r="F163" s="14"/>
       <c r="G163" s="14"/>
@@ -27548,7 +27550,7 @@
       <c r="D170" s="58"/>
       <c r="E170" s="92">
         <f ca="1">E163</f>
-        <v>23088.56</v>
+        <v>23067.86</v>
       </c>
       <c r="F170" s="14"/>
       <c r="G170" s="14"/>
@@ -27820,7 +27822,7 @@
       <c r="D190" s="82"/>
       <c r="E190" s="92">
         <f ca="1">(F40+E170)-(SUM(E172:E181)+SUM(E183:E189))</f>
-        <v>23934.57</v>
+        <v>23913.87</v>
       </c>
       <c r="F190" s="14"/>
       <c r="G190" s="14"/>
@@ -28312,7 +28314,7 @@
       </c>
       <c r="C2" s="4" cm="1">
         <f ca="1" t="array" ref="C2">INDIRECT("'"&amp;Main!B9&amp;"'!$C$16")</f>
-        <v>78.22</v>
+        <v>57.52</v>
       </c>
       <c r="D2" s="4"/>
       <c r="E2" s="4"/>
@@ -28328,7 +28330,7 @@
       </c>
       <c r="C3" s="7">
         <f ca="1">E190</f>
-        <v>25820.6</v>
+        <v>25799.9</v>
       </c>
       <c r="D3" s="7"/>
       <c r="E3" s="7"/>
@@ -28344,7 +28346,7 @@
       <c r="B4" s="9"/>
       <c r="C4" s="10">
         <f ca="1">SUM(C2:G3)</f>
-        <v>25898.82</v>
+        <v>25857.42</v>
       </c>
       <c r="D4" s="10"/>
       <c r="E4" s="10"/>
@@ -30164,7 +30166,7 @@
       <c r="D116" s="58"/>
       <c r="E116" s="71" cm="1">
         <f ca="1" t="array" ref="E116">INDIRECT("'"&amp;INDIRECT("Main!B48")&amp;"'!E190")</f>
-        <v>23934.57</v>
+        <v>23913.87</v>
       </c>
       <c r="F116" s="14"/>
       <c r="G116" s="14"/>
@@ -30436,7 +30438,7 @@
       <c r="D136" s="82"/>
       <c r="E136" s="89">
         <f ca="1">(F16+E116)-(SUM(E118:E127)+SUM(E129:E135))</f>
-        <v>24559.58</v>
+        <v>24538.88</v>
       </c>
       <c r="F136" s="14"/>
       <c r="G136" s="14"/>
@@ -30528,7 +30530,7 @@
       <c r="D143" s="58"/>
       <c r="E143" s="89">
         <f ca="1">E136</f>
-        <v>24559.58</v>
+        <v>24538.88</v>
       </c>
       <c r="F143" s="14"/>
       <c r="G143" s="14"/>
@@ -30800,7 +30802,7 @@
       <c r="D163" s="82"/>
       <c r="E163" s="92">
         <f ca="1">(F28+E143)-(SUM(E145:E154)+SUM(E156:E162))</f>
-        <v>25245.59</v>
+        <v>25224.89</v>
       </c>
       <c r="F163" s="14"/>
       <c r="G163" s="14"/>
@@ -30892,7 +30894,7 @@
       <c r="D170" s="58"/>
       <c r="E170" s="92">
         <f ca="1">E163</f>
-        <v>25245.59</v>
+        <v>25224.89</v>
       </c>
       <c r="F170" s="14"/>
       <c r="G170" s="14"/>
@@ -31164,7 +31166,7 @@
       <c r="D190" s="82"/>
       <c r="E190" s="92">
         <f ca="1">(F40+E170)-(SUM(E172:E181)+SUM(E183:E189))</f>
-        <v>25820.6</v>
+        <v>25799.9</v>
       </c>
       <c r="F190" s="14"/>
       <c r="G190" s="14"/>
@@ -31663,7 +31665,7 @@
       </c>
       <c r="C2" s="4" cm="1">
         <f ca="1" t="array" ref="C2">INDIRECT("'"&amp;Main!B9&amp;"'!$C$16")</f>
-        <v>78.22</v>
+        <v>57.52</v>
       </c>
       <c r="D2" s="4"/>
       <c r="E2" s="4"/>
@@ -31679,7 +31681,7 @@
       </c>
       <c r="C3" s="7">
         <f ca="1">E190</f>
-        <v>27927.63</v>
+        <v>27906.93</v>
       </c>
       <c r="D3" s="7"/>
       <c r="E3" s="7"/>
@@ -31695,7 +31697,7 @@
       <c r="B4" s="9"/>
       <c r="C4" s="10">
         <f ca="1">SUM(C2:G3)</f>
-        <v>28005.85</v>
+        <v>27964.45</v>
       </c>
       <c r="D4" s="10"/>
       <c r="E4" s="10"/>
@@ -33516,7 +33518,7 @@
       <c r="D116" s="58"/>
       <c r="E116" s="71" cm="1">
         <f ca="1" t="array" ref="E116">INDIRECT("'"&amp;INDIRECT("Main!B51")&amp;"'!E190")</f>
-        <v>25820.6</v>
+        <v>25799.9</v>
       </c>
       <c r="F116" s="14"/>
       <c r="G116" s="14"/>
@@ -33788,7 +33790,7 @@
       <c r="D136" s="82"/>
       <c r="E136" s="89">
         <f ca="1">(F16+E116)-(SUM(E118:E127)+SUM(E129:E135))</f>
-        <v>26666.61</v>
+        <v>26645.91</v>
       </c>
       <c r="F136" s="14"/>
       <c r="G136" s="14"/>
@@ -33880,7 +33882,7 @@
       <c r="D143" s="58"/>
       <c r="E143" s="89">
         <f ca="1">E136</f>
-        <v>26666.61</v>
+        <v>26645.91</v>
       </c>
       <c r="F143" s="14"/>
       <c r="G143" s="14"/>
@@ -34152,7 +34154,7 @@
       <c r="D163" s="82"/>
       <c r="E163" s="92">
         <f ca="1">(F28+E143)-(SUM(E145:E154)+SUM(E156:E162))</f>
-        <v>27081.62</v>
+        <v>27060.92</v>
       </c>
       <c r="F163" s="14"/>
       <c r="G163" s="14"/>
@@ -34244,7 +34246,7 @@
       <c r="D170" s="58"/>
       <c r="E170" s="92">
         <f ca="1">E163</f>
-        <v>27081.62</v>
+        <v>27060.92</v>
       </c>
       <c r="F170" s="14"/>
       <c r="G170" s="14"/>
@@ -34516,7 +34518,7 @@
       <c r="D190" s="82"/>
       <c r="E190" s="92">
         <f ca="1">(F40+E170)-(SUM(E172:E181)+SUM(E183:E189))</f>
-        <v>27927.63</v>
+        <v>27906.93</v>
       </c>
       <c r="F190" s="14"/>
       <c r="G190" s="14"/>
@@ -35579,7 +35581,7 @@
         <v>35</v>
       </c>
       <c r="C3" s="159">
-        <v>18.4</v>
+        <v>0.4</v>
       </c>
       <c r="D3" s="160" t="s">
         <v>34</v>
@@ -35692,7 +35694,7 @@
       </c>
       <c r="J6" s="196">
         <f ca="1">'April 2025 - June 2025'!E136</f>
-        <v>78.22</v>
+        <v>57.52</v>
       </c>
       <c r="M6" s="201" t="str">
         <f>IF(Main!B2,TEXT(EDATE(Main!B3,9),"dd mmmm yyyy"),TEXT(Main!B3+((Main!B5-Main!B3)*9+9),"dd mmmm yyyy"))&amp;" - "&amp;IF(Main!B2,TEXT(EDATE(Main!B3,12)-1,"dd mmmm yyyy"),TEXT(Main!B3+((Main!B5-Main!B3)*12+11),"dd mmmm yyyy"))</f>
@@ -35724,7 +35726,7 @@
       </c>
       <c r="J7" s="196">
         <f ca="1">'April 2025 - June 2025'!E163</f>
-        <v>304.23</v>
+        <v>283.53</v>
       </c>
       <c r="M7" s="201" t="str">
         <f>IF(Main!B2,TEXT(EDATE(Main!B3,12),"dd mmmm yyyy"),TEXT(Main!B3+((Main!B5-Main!B3)*12+12),"dd mmmm yyyy"))&amp;" - "&amp;IF(Main!B2,TEXT(EDATE(Main!B3,15)-1,"dd mmmm yyyy"),TEXT(Main!B3+((Main!B5-Main!B3)*15+14),"dd mmmm yyyy"))</f>
@@ -35757,7 +35759,7 @@
       </c>
       <c r="J8" s="196">
         <f ca="1">'April 2025 - June 2025'!E190</f>
-        <v>259.240000000001</v>
+        <v>238.54</v>
       </c>
       <c r="M8" s="204" t="str">
         <f>IF(Main!B2,TEXT(EDATE(Main!B3,15),"dd mmmm yyyy"),TEXT(Main!B3+((Main!B5-Main!B3)*15+15),"dd mmmm yyyy"))&amp;" - "&amp;IF(Main!B2,TEXT(EDATE(Main!B3,18)-1,"dd mmmm yyyy"),TEXT(Main!B3+((Main!B5-Main!B3)*18+17),"dd mmmm yyyy"))</f>
@@ -35789,7 +35791,7 @@
       </c>
       <c r="J9" s="196">
         <f ca="1">'July 2025 - September 2025'!E136</f>
-        <v>305.250000000001</v>
+        <v>284.550000000001</v>
       </c>
       <c r="M9" s="201" t="str">
         <f>IF(Main!B2,TEXT(EDATE(Main!B3,18),"dd mmmm yyyy"),TEXT(Main!B3+((Main!B5-Main!B3)*18+18),"dd mmmm yyyy"))&amp;" - "&amp;IF(Main!B2,TEXT(EDATE(Main!B3,21)-1,"dd mmmm yyyy"),TEXT(Main!B3+((Main!B5-Main!B3)*21+20),"dd mmmm yyyy"))</f>
@@ -35821,7 +35823,7 @@
       </c>
       <c r="J10" s="196">
         <f ca="1">'July 2025 - September 2025'!E163</f>
-        <v>210.260000000001</v>
+        <v>189.560000000001</v>
       </c>
       <c r="M10" s="206" t="str">
         <f>IF(Main!B2,TEXT(EDATE(Main!B3,21),"dd mmmm yyyy"),TEXT(Main!B3+((Main!B5-Main!B3)*21+21),"dd mmmm yyyy"))&amp;" - "&amp;IF(Main!B2,TEXT(EDATE(Main!B3,24)-1,"dd mmmm yyyy"),TEXT(Main!B3+((Main!B5-Main!B3)*24+23),"dd mmmm yyyy"))</f>
@@ -35838,14 +35840,14 @@
         <v>43</v>
       </c>
       <c r="C11" s="159">
-        <v>21.4</v>
+        <v>0</v>
       </c>
       <c r="D11" s="161"/>
       <c r="E11" s="5" t="s">
         <v>43</v>
       </c>
       <c r="F11" s="187">
-        <v>19.4</v>
+        <v>21.4</v>
       </c>
       <c r="H11" s="188"/>
       <c r="I11" s="197" t="str">
@@ -35854,7 +35856,7 @@
       </c>
       <c r="J11" s="196">
         <f ca="1">'July 2025 - September 2025'!E190</f>
-        <v>256.270000000001</v>
+        <v>235.570000000001</v>
       </c>
       <c r="M11" s="201" t="str">
         <f>IF(Main!B2,TEXT(EDATE(Main!B3,24),"dd mmmm yyyy"),TEXT(Main!B3+((Main!B5-Main!B3)*24+24),"dd mmmm yyyy"))&amp;" - "&amp;IF(Main!B2,TEXT(EDATE(Main!B3,27)-1,"dd mmmm yyyy"),TEXT(Main!B3+((Main!B5-Main!B3)*27+26),"dd mmmm yyyy"))</f>
@@ -35886,7 +35888,7 @@
       </c>
       <c r="J12" s="196">
         <f ca="1">'October 2025 - December 2025'!E136</f>
-        <v>211.280000000002</v>
+        <v>190.580000000001</v>
       </c>
       <c r="M12" s="197" t="str">
         <f>IF(Main!B2,TEXT(EDATE(Main!B3,27),"dd mmmm yyyy"),TEXT(Main!B3+((Main!B5-Main!B3)*27+27),"dd mmmm yyyy"))&amp;" - "&amp;IF(Main!B2,TEXT(EDATE(Main!B3,30)-1,"dd mmmm yyyy"),TEXT(Main!B3+((Main!B5-Main!B3)*30+29),"dd mmmm yyyy"))</f>
@@ -35918,7 +35920,7 @@
       </c>
       <c r="J13" s="196">
         <f ca="1">'October 2025 - December 2025'!E163</f>
-        <v>207.290000000002</v>
+        <v>186.590000000002</v>
       </c>
       <c r="M13" s="197" t="str">
         <f>IF(Main!B2,TEXT(EDATE(Main!B3,30),"dd mmmm yyyy"),TEXT(Main!B3+((Main!B5-Main!B3)*30+30),"dd mmmm yyyy"))&amp;" - "&amp;IF(Main!B2,TEXT(EDATE(Main!B3,33)-1,"dd mmmm yyyy"),TEXT(Main!B3+((Main!B5-Main!B3)*33+32),"dd mmmm yyyy"))</f>
@@ -35935,7 +35937,7 @@
         <v>46</v>
       </c>
       <c r="C14" s="159">
-        <v>7.4</v>
+        <v>26.1</v>
       </c>
       <c r="D14" s="161"/>
       <c r="E14" s="189" t="s">
@@ -35950,7 +35952,7 @@
       </c>
       <c r="J14" s="200">
         <f ca="1">'October 2025 - December 2025'!E190</f>
-        <v>132.300000000002</v>
+        <v>111.600000000002</v>
       </c>
       <c r="M14" s="197" t="str">
         <f>IF(Main!B2,TEXT(EDATE(Main!B3,33),"dd mmmm yyyy"),TEXT(Main!B3+((Main!B5-Main!B3)*33+33),"dd mmmm yyyy"))&amp;" - "&amp;IF(Main!B2,TEXT(EDATE(Main!B3,36)-1,"dd mmmm yyyy"),TEXT(Main!B3+((Main!B5-Main!B3)*36+35),"dd mmmm yyyy"))</f>
@@ -35982,7 +35984,7 @@
       </c>
       <c r="J15" s="200">
         <f ca="1">'January 2026 - March 2026'!E136</f>
-        <v>295.310000000002</v>
+        <v>274.610000000002</v>
       </c>
       <c r="M15" s="197" t="str">
         <f>IF(Main!B2,TEXT(EDATE(Main!B3,36),"dd mmmm yyyy"),TEXT(Main!B3+((Main!B5-Main!B3)*36+36),"dd mmmm yyyy"))&amp;" - "&amp;IF(Main!B2,TEXT(EDATE(Main!B3,39)-1,"dd mmmm yyyy"),TEXT(Main!B3+((Main!B5-Main!B3)*39+38),"dd mmmm yyyy"))</f>
@@ -36000,7 +36002,7 @@
       </c>
       <c r="C16" s="165">
         <f>SUM(C3:C15)</f>
-        <v>78.22</v>
+        <v>57.52</v>
       </c>
       <c r="D16" s="166"/>
       <c r="E16" s="164" t="s">
@@ -36008,7 +36010,7 @@
       </c>
       <c r="F16" s="190">
         <f>SUM(F3:F15)</f>
-        <v>76.22</v>
+        <v>78.22</v>
       </c>
       <c r="I16" s="201" t="str">
         <f>IF(Main!B2,TEXT(EDATE(Main!B3,13),"dd mmmm yyyy"),TEXT(Main!B3+((Main!B5-Main!B3)*13)+13,"dd mmmm yyyy"))&amp;" - "&amp;IF(Main!B2,TEXT(EDATE(Main!B3,14)-1,"dd mmmm yyyy"),TEXT(Main!B3+((Main!B5-Main!B3)*14+13),"dd mmmm yyyy"))</f>
@@ -36016,7 +36018,7 @@
       </c>
       <c r="J16" s="200">
         <f ca="1">'January 2026 - March 2026'!E163</f>
-        <v>710.320000000002</v>
+        <v>689.620000000002</v>
       </c>
       <c r="M16" s="197" t="str">
         <f>IF(Main!B2,TEXT(EDATE(Main!B3,39),"dd mmmm yyyy"),TEXT(Main!B3+((Main!B5-Main!B3)*39+39),"dd mmmm yyyy"))&amp;" - "&amp;IF(Main!B2,TEXT(EDATE(Main!B3,42)-1,"dd mmmm yyyy"),TEXT(Main!B3+((Main!B5-Main!B3)*42+41),"dd mmmm yyyy"))</f>
@@ -36034,7 +36036,7 @@
       </c>
       <c r="J17" s="200">
         <f ca="1">'January 2026 - March 2026'!E190</f>
-        <v>1556.33</v>
+        <v>1535.63</v>
       </c>
       <c r="M17" s="197" t="str">
         <f>IF(Main!B2,TEXT(EDATE(Main!B3,42),"dd mmmm yyyy"),TEXT(Main!B3+((Main!B5-Main!B3)*42+42),"dd mmmm yyyy"))&amp;" - "&amp;IF(Main!B2,TEXT(EDATE(Main!B3,45)-1,"dd mmmm yyyy"),TEXT(Main!B3+((Main!B5-Main!B3)*45+44),"dd mmmm yyyy"))</f>
@@ -36052,7 +36054,7 @@
       </c>
       <c r="J18" s="200">
         <f ca="1">'April 2026 - June 2026'!E136</f>
-        <v>2131.34</v>
+        <v>2110.64</v>
       </c>
       <c r="M18" s="197" t="str">
         <f>IF(Main!B2,TEXT(EDATE(Main!B3,45),"dd mmmm yyyy"),TEXT(Main!B3+((Main!B5-Main!B3)*45+45),"dd mmmm yyyy"))&amp;" - "&amp;IF(Main!B2,TEXT(EDATE(Main!B3,48)-1,"dd mmmm yyyy"),TEXT(Main!B3+((Main!B5-Main!B3)*48+47),"dd mmmm yyyy"))</f>
@@ -36070,7 +36072,7 @@
       </c>
       <c r="J19" s="200">
         <f ca="1">'April 2026 - June 2026'!E163</f>
-        <v>3900.35</v>
+        <v>3879.65</v>
       </c>
     </row>
     <row r="20" ht="35.25" customHeight="1" spans="9:10">
@@ -36080,7 +36082,7 @@
       </c>
       <c r="J20" s="200">
         <f ca="1">'April 2026 - June 2026'!E190</f>
-        <v>4525.36</v>
+        <v>4504.66</v>
       </c>
     </row>
     <row r="21" ht="35.25" customHeight="1" spans="9:10">
@@ -36090,7 +36092,7 @@
       </c>
       <c r="J21" s="200">
         <f ca="1">'July 2026 - September 2026'!E136</f>
-        <v>5371.37</v>
+        <v>5350.67</v>
       </c>
     </row>
     <row r="22" ht="24.75" customHeight="1" spans="1:10">
@@ -36110,7 +36112,7 @@
       </c>
       <c r="J22" s="200">
         <f ca="1">'July 2026 - September 2026'!E163</f>
-        <v>5786.38</v>
+        <v>5765.68</v>
       </c>
     </row>
     <row r="23" ht="24.75" customHeight="1" spans="1:10">
@@ -36135,7 +36137,7 @@
       </c>
       <c r="J23" s="200">
         <f ca="1">'July 2026 - September 2026'!E190</f>
-        <v>6632.39</v>
+        <v>6611.69</v>
       </c>
     </row>
     <row r="24" ht="33" customHeight="1" spans="1:10">
@@ -36154,7 +36156,7 @@
       </c>
       <c r="J24" s="200">
         <f ca="1">'October 2026 - December 2026'!E136</f>
-        <v>7207.40000000001</v>
+        <v>7186.7</v>
       </c>
     </row>
     <row r="25" ht="30" customHeight="1" spans="1:10">
@@ -36173,7 +36175,7 @@
       </c>
       <c r="J25" s="200">
         <f ca="1">'October 2026 - December 2026'!E163</f>
-        <v>7893.41000000001</v>
+        <v>7872.71</v>
       </c>
     </row>
     <row r="26" ht="30" customHeight="1" spans="1:10">
@@ -36192,7 +36194,7 @@
       </c>
       <c r="J26" s="200">
         <f ca="1">'October 2026 - December 2026'!E190</f>
-        <v>8468.42000000001</v>
+        <v>8447.72</v>
       </c>
     </row>
     <row r="27" ht="30" customHeight="1" spans="1:10">
@@ -36211,7 +36213,7 @@
       </c>
       <c r="J27" s="200">
         <f ca="1">'January 2027 - March 2027'!E136</f>
-        <v>9314.43000000001</v>
+        <v>9293.73</v>
       </c>
     </row>
     <row r="28" ht="30" customHeight="1" spans="1:10">
@@ -36230,7 +36232,7 @@
       </c>
       <c r="J28" s="200">
         <f ca="1">'January 2027 - March 2027'!E163</f>
-        <v>9729.44000000001</v>
+        <v>9708.74000000001</v>
       </c>
     </row>
     <row r="29" ht="30" customHeight="1" spans="1:10">
@@ -36249,7 +36251,7 @@
       </c>
       <c r="J29" s="196">
         <f ca="1">'January 2027 - March 2027'!E190</f>
-        <v>10575.45</v>
+        <v>10554.75</v>
       </c>
     </row>
     <row r="30" ht="30" customHeight="1" spans="1:10">
@@ -36271,7 +36273,7 @@
       </c>
       <c r="J30" s="202">
         <f ca="1">'April 2027 - June 2027'!E136</f>
-        <v>11791.45</v>
+        <v>11770.75</v>
       </c>
     </row>
     <row r="31" ht="30" customHeight="1" spans="9:10">
@@ -36281,7 +36283,7 @@
       </c>
       <c r="J31" s="200">
         <f ca="1">'April 2027 - June 2027'!E163</f>
-        <v>13659.45</v>
+        <v>13638.75</v>
       </c>
     </row>
     <row r="32" ht="27.75" customHeight="1" spans="9:10">
@@ -36291,7 +36293,7 @@
       </c>
       <c r="J32" s="200">
         <f ca="1">'April 2027 - June 2027'!E190</f>
-        <v>14875.45</v>
+        <v>14854.75</v>
       </c>
     </row>
     <row r="33" ht="30" customHeight="1" spans="9:10">
@@ -36301,7 +36303,7 @@
       </c>
       <c r="J33" s="200">
         <f ca="1">'July 2027 - September 2027'!E136</f>
-        <v>15450.46</v>
+        <v>15429.76</v>
       </c>
     </row>
     <row r="34" ht="30" customHeight="1" spans="1:10">
@@ -36321,7 +36323,7 @@
       </c>
       <c r="J34" s="200">
         <f ca="1">'July 2027 - September 2027'!E163</f>
-        <v>16136.47</v>
+        <v>16115.77</v>
       </c>
     </row>
     <row r="35" ht="24.75" customHeight="1" spans="1:10">
@@ -36346,7 +36348,7 @@
       </c>
       <c r="J35" s="200">
         <f ca="1">'July 2027 - September 2027'!E190</f>
-        <v>16711.48</v>
+        <v>16690.78</v>
       </c>
     </row>
     <row r="36" ht="22" customHeight="1" spans="1:10">
@@ -36369,7 +36371,7 @@
       </c>
       <c r="J36" s="200">
         <f ca="1">'October 2027 - December 2027'!E136</f>
-        <v>17557.49</v>
+        <v>17536.79</v>
       </c>
     </row>
     <row r="37" ht="24.75" customHeight="1" spans="1:10">
@@ -36388,7 +36390,7 @@
       </c>
       <c r="J37" s="200">
         <f ca="1">'October 2027 - December 2027'!E163</f>
-        <v>17972.5</v>
+        <v>17951.8</v>
       </c>
     </row>
     <row r="38" ht="20.25" customHeight="1" spans="1:10">
@@ -36407,7 +36409,7 @@
       </c>
       <c r="J38" s="200">
         <f ca="1">'October 2027 - December 2027'!E190</f>
-        <v>18818.51</v>
+        <v>18797.81</v>
       </c>
     </row>
     <row r="39" ht="24.75" customHeight="1" spans="1:10">
@@ -36426,7 +36428,7 @@
       </c>
       <c r="J39" s="200">
         <f ca="1">'January 2028 - March 2028'!E136</f>
-        <v>19443.52</v>
+        <v>19422.82</v>
       </c>
     </row>
     <row r="40" ht="24.75" customHeight="1" spans="1:10">
@@ -36445,7 +36447,7 @@
       </c>
       <c r="J40" s="200">
         <f ca="1">'January 2028 - March 2028'!E163</f>
-        <v>20129.53</v>
+        <v>20108.83</v>
       </c>
     </row>
     <row r="41" ht="24.75" customHeight="1" spans="1:10">
@@ -36464,7 +36466,7 @@
       </c>
       <c r="J41" s="200">
         <f ca="1">'January 2028 - March 2028'!E190</f>
-        <v>20744.54</v>
+        <v>20723.84</v>
       </c>
     </row>
     <row r="42" ht="24.75" customHeight="1" spans="1:10">
@@ -36486,7 +36488,7 @@
       </c>
       <c r="J42" s="200">
         <f ca="1">'April 2028 - June 2028'!E136</f>
-        <v>21590.55</v>
+        <v>21569.85</v>
       </c>
     </row>
     <row r="43" ht="24.75" customHeight="1" spans="9:10">
@@ -36496,7 +36498,7 @@
       </c>
       <c r="J43" s="200">
         <f ca="1">'April 2028 - June 2028'!E163</f>
-        <v>23088.56</v>
+        <v>23067.86</v>
       </c>
     </row>
     <row r="44" ht="24.75" customHeight="1" spans="9:10">
@@ -36506,7 +36508,7 @@
       </c>
       <c r="J44" s="200">
         <f ca="1">'April 2028 - June 2028'!E190</f>
-        <v>23934.57</v>
+        <v>23913.87</v>
       </c>
     </row>
     <row r="45" ht="24.75" customHeight="1" spans="9:10">
@@ -36516,7 +36518,7 @@
       </c>
       <c r="J45" s="200">
         <f ca="1">'July 2028 - September 2028'!E136</f>
-        <v>24559.58</v>
+        <v>24538.88</v>
       </c>
     </row>
     <row r="46" ht="24.75" customHeight="1" spans="1:10">
@@ -36536,7 +36538,7 @@
       </c>
       <c r="J46" s="200">
         <f ca="1">'July 2028 - September 2028'!E163</f>
-        <v>25245.59</v>
+        <v>25224.89</v>
       </c>
     </row>
     <row r="47" ht="24.75" customHeight="1" spans="1:10">
@@ -36561,7 +36563,7 @@
       </c>
       <c r="J47" s="200">
         <f ca="1">'July 2028 - September 2028'!E190</f>
-        <v>25820.6</v>
+        <v>25799.9</v>
       </c>
     </row>
     <row r="48" ht="24.75" customHeight="1" spans="1:10">
@@ -36584,7 +36586,7 @@
       </c>
       <c r="J48" s="200">
         <f ca="1">'October 2028 - December 2028'!E136</f>
-        <v>26666.61</v>
+        <v>26645.91</v>
       </c>
     </row>
     <row r="49" ht="24.75" customHeight="1" spans="1:10">
@@ -36603,7 +36605,7 @@
       </c>
       <c r="J49" s="200">
         <f ca="1">'October 2028 - December 2028'!E163</f>
-        <v>27081.62</v>
+        <v>27060.92</v>
       </c>
     </row>
     <row r="50" ht="24.75" customHeight="1" spans="1:10">
@@ -36622,7 +36624,7 @@
       </c>
       <c r="J50" s="196">
         <f ca="1">'October 2028 - December 2028'!E190</f>
-        <v>27927.63</v>
+        <v>27906.93</v>
       </c>
     </row>
     <row r="51" ht="41.1" customHeight="1" spans="1:7">
@@ -38519,7 +38521,7 @@
       </c>
       <c r="C2" s="4" cm="1">
         <f ca="1" t="array" ref="C2">INDIRECT("'"&amp;Main!B9&amp;"'!$C$16")</f>
-        <v>78.22</v>
+        <v>57.52</v>
       </c>
       <c r="D2" s="4"/>
       <c r="E2" s="4"/>
@@ -38533,7 +38535,7 @@
       </c>
       <c r="C3" s="7">
         <f ca="1">E190</f>
-        <v>259.240000000001</v>
+        <v>238.54</v>
       </c>
       <c r="D3" s="7"/>
       <c r="E3" s="7"/>
@@ -38547,7 +38549,7 @@
       <c r="B4" s="9"/>
       <c r="C4" s="10">
         <f ca="1">SUM(C2:G3)</f>
-        <v>337.460000000001</v>
+        <v>296.06</v>
       </c>
       <c r="D4" s="10"/>
       <c r="E4" s="10"/>
@@ -40560,7 +40562,7 @@
       <c r="H128" s="14"/>
       <c r="I128" s="48"/>
     </row>
-    <row r="129" ht="40.5" customHeight="1" spans="1:9">
+    <row r="129" ht="59" customHeight="1" spans="1:9">
       <c r="A129" s="63"/>
       <c r="B129" s="64"/>
       <c r="C129" s="73" t="s">
@@ -40575,7 +40577,7 @@
       <c r="H129" s="14"/>
       <c r="I129" s="48"/>
     </row>
-    <row r="130" ht="153" customHeight="1" spans="1:9">
+    <row r="130" ht="186" customHeight="1" spans="1:9">
       <c r="A130" s="63"/>
       <c r="B130" s="64"/>
       <c r="C130" s="73" t="s">
@@ -40583,7 +40585,7 @@
       </c>
       <c r="D130" s="74"/>
       <c r="E130" s="87">
-        <v>603.5</v>
+        <v>624.2</v>
       </c>
       <c r="F130" s="14"/>
       <c r="G130" s="14"/>
@@ -40667,7 +40669,7 @@
       <c r="D136" s="82"/>
       <c r="E136" s="89">
         <f ca="1">(F16+E116)-(SUM(E118:E127)+SUM(E129:E135))</f>
-        <v>78.22</v>
+        <v>57.52</v>
       </c>
       <c r="F136" s="14"/>
       <c r="G136" s="14"/>
@@ -40759,7 +40761,7 @@
       <c r="D143" s="58"/>
       <c r="E143" s="89">
         <f ca="1">E136</f>
-        <v>78.22</v>
+        <v>57.52</v>
       </c>
       <c r="F143" s="14"/>
       <c r="G143" s="14"/>
@@ -41037,7 +41039,7 @@
       <c r="D163" s="82"/>
       <c r="E163" s="92">
         <f ca="1">(F28+E143)-(SUM(E145:E154)+SUM(E156:E162))</f>
-        <v>304.23</v>
+        <v>283.53</v>
       </c>
       <c r="F163" s="14"/>
       <c r="G163" s="14"/>
@@ -41128,7 +41130,7 @@
       <c r="D170" s="58"/>
       <c r="E170" s="92">
         <f ca="1">E163</f>
-        <v>304.23</v>
+        <v>283.53</v>
       </c>
       <c r="F170" s="14"/>
       <c r="G170" s="14"/>
@@ -41402,7 +41404,7 @@
       <c r="D190" s="82"/>
       <c r="E190" s="92">
         <f ca="1">(F40+E170)-(SUM(E172:E181)+SUM(E183:E189))</f>
-        <v>259.240000000001</v>
+        <v>238.54</v>
       </c>
       <c r="F190" s="14"/>
       <c r="G190" s="14"/>
@@ -41913,7 +41915,7 @@
       </c>
       <c r="C2" s="4" cm="1">
         <f ca="1" t="array" ref="C2">INDIRECT("'"&amp;Main!B9&amp;"'!$C$16")</f>
-        <v>78.22</v>
+        <v>57.52</v>
       </c>
       <c r="D2" s="4"/>
       <c r="E2" s="4"/>
@@ -41927,7 +41929,7 @@
       </c>
       <c r="C3" s="7">
         <f ca="1">E190</f>
-        <v>256.270000000001</v>
+        <v>235.570000000001</v>
       </c>
       <c r="D3" s="7"/>
       <c r="E3" s="7"/>
@@ -41941,7 +41943,7 @@
       <c r="B4" s="9"/>
       <c r="C4" s="10">
         <f ca="1">SUM(C2:G3)</f>
-        <v>334.490000000001</v>
+        <v>293.090000000001</v>
       </c>
       <c r="D4" s="10"/>
       <c r="E4" s="10"/>
@@ -43762,7 +43764,7 @@
       <c r="D116" s="58"/>
       <c r="E116" s="89" cm="1">
         <f ca="1" t="array" ref="E116">INDIRECT("'"&amp;INDIRECT("Main!B12")&amp;"'!E190")</f>
-        <v>259.240000000001</v>
+        <v>238.54</v>
       </c>
       <c r="F116" s="14"/>
       <c r="G116" s="14"/>
@@ -44036,7 +44038,7 @@
       <c r="D136" s="82"/>
       <c r="E136" s="89">
         <f ca="1">(F16+E116)-(SUM(E118:E127)+SUM(E129:E135))</f>
-        <v>305.250000000001</v>
+        <v>284.550000000001</v>
       </c>
       <c r="F136" s="14"/>
       <c r="G136" s="14"/>
@@ -44128,7 +44130,7 @@
       <c r="D143" s="58"/>
       <c r="E143" s="89">
         <f ca="1">E136</f>
-        <v>305.250000000001</v>
+        <v>284.550000000001</v>
       </c>
       <c r="F143" s="14"/>
       <c r="G143" s="14"/>
@@ -44402,7 +44404,7 @@
       <c r="D163" s="82"/>
       <c r="E163" s="92">
         <f ca="1">(F28+E143)-(SUM(E145:E154)+SUM(E156:E162))</f>
-        <v>210.260000000001</v>
+        <v>189.560000000001</v>
       </c>
       <c r="F163" s="14"/>
       <c r="G163" s="14"/>
@@ -44494,7 +44496,7 @@
       <c r="D170" s="58"/>
       <c r="E170" s="92">
         <f ca="1">E163</f>
-        <v>210.260000000001</v>
+        <v>189.560000000001</v>
       </c>
       <c r="F170" s="14"/>
       <c r="G170" s="14"/>
@@ -44768,7 +44770,7 @@
       <c r="D190" s="82"/>
       <c r="E190" s="92">
         <f ca="1">(F40+E170)-(SUM(E172:E181)+SUM(E183:E189))</f>
-        <v>256.270000000001</v>
+        <v>235.570000000001</v>
       </c>
       <c r="F190" s="14"/>
       <c r="G190" s="14"/>
@@ -45328,7 +45330,7 @@
       </c>
       <c r="C2" s="4" cm="1">
         <f ca="1" t="array" ref="C2">INDIRECT("'"&amp;Main!B9&amp;"'!$C$16")</f>
-        <v>78.22</v>
+        <v>57.52</v>
       </c>
       <c r="D2" s="4"/>
       <c r="E2" s="4"/>
@@ -45344,7 +45346,7 @@
       </c>
       <c r="C3" s="7">
         <f ca="1">E190</f>
-        <v>132.300000000002</v>
+        <v>111.600000000002</v>
       </c>
       <c r="D3" s="7"/>
       <c r="E3" s="7"/>
@@ -45360,7 +45362,7 @@
       <c r="B4" s="9"/>
       <c r="C4" s="10">
         <f ca="1">SUM(C2:G3)</f>
-        <v>210.520000000002</v>
+        <v>169.120000000002</v>
       </c>
       <c r="D4" s="10"/>
       <c r="E4" s="10"/>
@@ -47181,7 +47183,7 @@
       <c r="D116" s="58"/>
       <c r="E116" s="71" cm="1">
         <f ca="1" t="array" ref="E116">INDIRECT("'"&amp;INDIRECT("Main!B15")&amp;"'!E190")</f>
-        <v>256.270000000001</v>
+        <v>235.570000000001</v>
       </c>
       <c r="F116" s="14"/>
       <c r="G116" s="14"/>
@@ -47455,7 +47457,7 @@
       <c r="D136" s="82"/>
       <c r="E136" s="89">
         <f ca="1">(F16+E116)-(SUM(E118:E127)+SUM(E129:E135))</f>
-        <v>211.280000000002</v>
+        <v>190.580000000001</v>
       </c>
       <c r="F136" s="14"/>
       <c r="G136" s="14"/>
@@ -47547,7 +47549,7 @@
       <c r="D143" s="58"/>
       <c r="E143" s="89">
         <f ca="1">E136</f>
-        <v>211.280000000002</v>
+        <v>190.580000000001</v>
       </c>
       <c r="F143" s="14"/>
       <c r="G143" s="14"/>
@@ -47821,7 +47823,7 @@
       <c r="D163" s="82"/>
       <c r="E163" s="92">
         <f ca="1">(F28+E143)-(SUM(E145:E154)+SUM(E156:E162))</f>
-        <v>207.290000000002</v>
+        <v>186.590000000002</v>
       </c>
       <c r="F163" s="14"/>
       <c r="G163" s="14"/>
@@ -47913,7 +47915,7 @@
       <c r="D170" s="58"/>
       <c r="E170" s="92">
         <f ca="1">E163</f>
-        <v>207.290000000002</v>
+        <v>186.590000000002</v>
       </c>
       <c r="F170" s="14"/>
       <c r="G170" s="14"/>
@@ -48189,7 +48191,7 @@
       <c r="D190" s="82"/>
       <c r="E190" s="92">
         <f ca="1">(F40+E170)-(SUM(E172:E181)+SUM(E183:E189))</f>
-        <v>132.300000000002</v>
+        <v>111.600000000002</v>
       </c>
       <c r="F190" s="14"/>
       <c r="G190" s="14"/>
@@ -48759,7 +48761,7 @@
       </c>
       <c r="C2" s="4" cm="1">
         <f ca="1" t="array" ref="C2">INDIRECT("'"&amp;Main!B9&amp;"'!$C$16")</f>
-        <v>78.22</v>
+        <v>57.52</v>
       </c>
       <c r="D2" s="4"/>
       <c r="E2" s="4"/>
@@ -48775,7 +48777,7 @@
       </c>
       <c r="C3" s="7">
         <f ca="1">E190</f>
-        <v>1556.33</v>
+        <v>1535.63</v>
       </c>
       <c r="D3" s="7"/>
       <c r="E3" s="7"/>
@@ -48791,7 +48793,7 @@
       <c r="B4" s="9"/>
       <c r="C4" s="10">
         <f ca="1">SUM(C2:G3)</f>
-        <v>1634.55</v>
+        <v>1593.15</v>
       </c>
       <c r="D4" s="10"/>
       <c r="E4" s="10"/>
@@ -50612,7 +50614,7 @@
       <c r="D116" s="58"/>
       <c r="E116" s="71" cm="1">
         <f ca="1" t="array" ref="E116">INDIRECT("'"&amp;INDIRECT("Main!B18")&amp;"'!E190")</f>
-        <v>132.300000000002</v>
+        <v>111.600000000002</v>
       </c>
       <c r="F116" s="14"/>
       <c r="G116" s="14"/>
@@ -50886,7 +50888,7 @@
       <c r="D136" s="82"/>
       <c r="E136" s="89">
         <f ca="1">(F16+E116)-(SUM(E118:E127)+SUM(E129:E135))</f>
-        <v>295.310000000002</v>
+        <v>274.610000000002</v>
       </c>
       <c r="F136" s="14"/>
       <c r="G136" s="14"/>
@@ -50978,7 +50980,7 @@
       <c r="D143" s="58"/>
       <c r="E143" s="89">
         <f ca="1">E136</f>
-        <v>295.310000000002</v>
+        <v>274.610000000002</v>
       </c>
       <c r="F143" s="14"/>
       <c r="G143" s="14"/>
@@ -51250,7 +51252,7 @@
       <c r="D163" s="82"/>
       <c r="E163" s="92">
         <f ca="1">(F28+E143)-(SUM(E145:E154)+SUM(E156:E162))</f>
-        <v>710.320000000002</v>
+        <v>689.620000000002</v>
       </c>
       <c r="F163" s="14"/>
       <c r="G163" s="14"/>
@@ -51342,7 +51344,7 @@
       <c r="D170" s="58"/>
       <c r="E170" s="92">
         <f ca="1">E163</f>
-        <v>710.320000000002</v>
+        <v>689.620000000002</v>
       </c>
       <c r="F170" s="14"/>
       <c r="G170" s="14"/>
@@ -51614,7 +51616,7 @@
       <c r="D190" s="82"/>
       <c r="E190" s="92">
         <f ca="1">(F40+E170)-(SUM(E172:E181)+SUM(E183:E189))</f>
-        <v>1556.33</v>
+        <v>1535.63</v>
       </c>
       <c r="F190" s="14"/>
       <c r="G190" s="14"/>
@@ -52142,7 +52144,7 @@
       </c>
       <c r="C2" s="4" cm="1">
         <f ca="1" t="array" ref="C2">INDIRECT("'"&amp;Main!B9&amp;"'!$C$16")</f>
-        <v>78.22</v>
+        <v>57.52</v>
       </c>
       <c r="D2" s="4"/>
       <c r="E2" s="4"/>
@@ -52158,7 +52160,7 @@
       </c>
       <c r="C3" s="7">
         <f ca="1">E190</f>
-        <v>4525.36</v>
+        <v>4504.66</v>
       </c>
       <c r="D3" s="7"/>
       <c r="E3" s="7"/>
@@ -52174,7 +52176,7 @@
       <c r="B4" s="9"/>
       <c r="C4" s="10">
         <f ca="1">SUM(C2:G3)</f>
-        <v>4603.58</v>
+        <v>4562.18</v>
       </c>
       <c r="D4" s="10"/>
       <c r="E4" s="10"/>
@@ -53999,7 +54001,7 @@
       <c r="D116" s="58"/>
       <c r="E116" s="71" cm="1">
         <f ca="1" t="array" ref="E116">INDIRECT("'"&amp;INDIRECT("Main!B21")&amp;"'!E190")</f>
-        <v>1556.33</v>
+        <v>1535.63</v>
       </c>
       <c r="F116" s="14"/>
       <c r="G116" s="14"/>
@@ -54271,7 +54273,7 @@
       <c r="D136" s="82"/>
       <c r="E136" s="89">
         <f ca="1">(F16+E116)-(SUM(E118:E127)+SUM(E129:E135))</f>
-        <v>2131.34</v>
+        <v>2110.64</v>
       </c>
       <c r="F136" s="14"/>
       <c r="G136" s="14"/>
@@ -54363,7 +54365,7 @@
       <c r="D143" s="58"/>
       <c r="E143" s="89">
         <f ca="1">E136</f>
-        <v>2131.34</v>
+        <v>2110.64</v>
       </c>
       <c r="F143" s="14"/>
       <c r="G143" s="14"/>
@@ -54635,7 +54637,7 @@
       <c r="D163" s="82"/>
       <c r="E163" s="92">
         <f ca="1">(F28+E143)-(SUM(E145:E154)+SUM(E156:E162))</f>
-        <v>3900.35</v>
+        <v>3879.65</v>
       </c>
       <c r="F163" s="14"/>
       <c r="G163" s="14"/>
@@ -54727,7 +54729,7 @@
       <c r="D170" s="58"/>
       <c r="E170" s="92">
         <f ca="1">E163</f>
-        <v>3900.35</v>
+        <v>3879.65</v>
       </c>
       <c r="F170" s="14"/>
       <c r="G170" s="14"/>
@@ -54999,7 +55001,7 @@
       <c r="D190" s="82"/>
       <c r="E190" s="92">
         <f ca="1">(F40+E170)-(SUM(E172:E181)+SUM(E183:E189))</f>
-        <v>4525.36</v>
+        <v>4504.66</v>
       </c>
       <c r="F190" s="14"/>
       <c r="G190" s="14"/>
@@ -55524,7 +55526,7 @@
       </c>
       <c r="C2" s="4" cm="1">
         <f ca="1" t="array" ref="C2">INDIRECT("'"&amp;Main!B9&amp;"'!$C$16")</f>
-        <v>78.22</v>
+        <v>57.52</v>
       </c>
       <c r="D2" s="4"/>
       <c r="E2" s="4"/>
@@ -55540,7 +55542,7 @@
       </c>
       <c r="C3" s="7">
         <f ca="1">E190</f>
-        <v>6632.39</v>
+        <v>6611.69</v>
       </c>
       <c r="D3" s="7"/>
       <c r="E3" s="7"/>
@@ -55556,7 +55558,7 @@
       <c r="B4" s="9"/>
       <c r="C4" s="10">
         <f ca="1">SUM(C2:G3)</f>
-        <v>6710.61000000001</v>
+        <v>6669.21</v>
       </c>
       <c r="D4" s="10"/>
       <c r="E4" s="10"/>
@@ -57379,7 +57381,7 @@
       <c r="D116" s="58"/>
       <c r="E116" s="71" cm="1">
         <f ca="1" t="array" ref="E116">INDIRECT("'"&amp;INDIRECT("Main!B24")&amp;"'!E190")</f>
-        <v>4525.36</v>
+        <v>4504.66</v>
       </c>
       <c r="F116" s="14"/>
       <c r="G116" s="14"/>
@@ -57651,7 +57653,7 @@
       <c r="D136" s="82"/>
       <c r="E136" s="89">
         <f ca="1">(F16+E116)-(SUM(E118:E127)+SUM(E129:E135))</f>
-        <v>5371.37</v>
+        <v>5350.67</v>
       </c>
       <c r="F136" s="14"/>
       <c r="G136" s="14"/>
@@ -57743,7 +57745,7 @@
       <c r="D143" s="58"/>
       <c r="E143" s="89">
         <f ca="1">E136</f>
-        <v>5371.37</v>
+        <v>5350.67</v>
       </c>
       <c r="F143" s="14"/>
       <c r="G143" s="14"/>
@@ -58015,7 +58017,7 @@
       <c r="D163" s="82"/>
       <c r="E163" s="92">
         <f ca="1">(F28+E143)-(SUM(E145:E154)+SUM(E156:E162))</f>
-        <v>5786.38</v>
+        <v>5765.68</v>
       </c>
       <c r="F163" s="14"/>
       <c r="G163" s="14"/>
@@ -58107,7 +58109,7 @@
       <c r="D170" s="58"/>
       <c r="E170" s="92">
         <f ca="1">E163</f>
-        <v>5786.38</v>
+        <v>5765.68</v>
       </c>
       <c r="F170" s="14"/>
       <c r="G170" s="14"/>
@@ -58379,7 +58381,7 @@
       <c r="D190" s="82"/>
       <c r="E190" s="92">
         <f ca="1">(F40+E170)-(SUM(E172:E181)+SUM(E183:E189))</f>
-        <v>6632.39</v>
+        <v>6611.69</v>
       </c>
       <c r="F190" s="14"/>
       <c r="G190" s="14"/>

</xml_diff>